<commit_message>
Sync templates from product/templates: store.json and its files
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EiAPcndz9mZ73fvAWuA5p3
</commit_message>
<xml_diff>
--- a/content/templates/files/first-sale-math/127-first-sale-math-example.xlsx
+++ b/content/templates/files/first-sale-math/127-first-sale-math-example.xlsx
@@ -639,7 +639,7 @@
     <row r="9" ht="16" customHeight="1">
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>1.  Open the Math tab. Fill the white cells for your test price in column B.</t>
+          <t>1.  Open the Math tab. Fill the white cells for your test price in column C.</t>
         </is>
       </c>
     </row>
@@ -667,7 +667,7 @@
     <row r="13" ht="16" customHeight="1">
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>5.  Try a lower and a higher price in columns C and D to compare.</t>
+          <t>5.  Try a lower and a higher price in columns B and D to compare.</t>
         </is>
       </c>
     </row>

</xml_diff>